<commit_message>
Fix AB summary overwrite in dashboard
</commit_message>
<xml_diff>
--- a/kpi_dashboard_with_charts.xlsx
+++ b/kpi_dashboard_with_charts.xlsx
@@ -11,7 +11,8 @@
     <sheet name="MAU_monthly" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Revenue_daily" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="AB_retention" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Dashboard" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="AB_summary" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Dashboard" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -21,18 +22,10 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
-      <color theme="1"/>
-      <sz val="11"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <b val="1"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
@@ -46,7 +39,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -54,30 +47,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -542,7 +517,7 @@
           <order val="0"/>
           <tx>
             <strRef>
-              <f>'AB_retention'!I1</f>
+              <f>'AB_summary'!B1</f>
             </strRef>
           </tx>
           <spPr>
@@ -552,12 +527,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'AB_retention'!$H$2:$H$4</f>
+              <f>'AB_summary'!$A$2:$A$4</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'AB_retention'!$I$2:$I$4</f>
+              <f>'AB_summary'!$B$2:$B$4</f>
             </numRef>
           </val>
         </ser>
@@ -1006,12 +981,12 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>day</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>dau</t>
         </is>
@@ -2842,12 +2817,12 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>week</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>wau</t>
         </is>
@@ -3138,12 +3113,12 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>month</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>mau</t>
         </is>
@@ -3259,12 +3234,12 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>day</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>revenue_eur</t>
         </is>
@@ -5095,52 +5070,52 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>experiment_name</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>variant</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>cohort_first_day</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>cohort_size</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>day1_active</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>day7_active</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>day30_active</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>variant</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>avg_d1_retention</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>d1_retention</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>d7_retention</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
         <is>
           <t>d30_retention</t>
         </is>
@@ -5174,14 +5149,11 @@
       <c r="G2" t="n">
         <v>526</v>
       </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>control</t>
-        </is>
-      </c>
-      <c r="I2">
-        <f>AVERAGEIF($B:$B,H2,$H:$H)</f>
-        <v/>
+      <c r="H2" t="n">
+        <v>0.02821645363470365</v>
+      </c>
+      <c r="I2" t="n">
+        <v>0.01284360657355772</v>
       </c>
       <c r="J2" t="n">
         <v>0.006489660958397078</v>
@@ -5215,14 +5187,11 @@
       <c r="G3" t="n">
         <v>528</v>
       </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="I3">
-        <f>AVERAGEIF($B:$B,H3,$H:$H)</f>
-        <v/>
+      <c r="H3" t="n">
+        <v>0.02368817662014933</v>
+      </c>
+      <c r="I3" t="n">
+        <v>0.01318438582160813</v>
       </c>
       <c r="J3" t="n">
         <v>0.006074481425662383</v>
@@ -5256,14 +5225,11 @@
       <c r="G4" t="n">
         <v>464</v>
       </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="I4">
-        <f>AVERAGEIF($B:$B,H4,$H:$H)</f>
-        <v/>
+      <c r="H4" t="n">
+        <v>0.01674130008487722</v>
+      </c>
+      <c r="I4" t="n">
+        <v>0.01366815933503088</v>
       </c>
       <c r="J4" t="n">
         <v>0.006790177656803348</v>
@@ -25800,6 +25766,62 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:B4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>variant</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>avg_d1_retention</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Control</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>0.03133003009976514</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>0.03250071151041475</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>0.03189500585796919</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:A1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>

</xml_diff>

<commit_message>
Increase chart title font sizes safely
</commit_message>
<xml_diff>
--- a/kpi_dashboard_with_charts.xlsx
+++ b/kpi_dashboard_with_charts.xlsx
@@ -165,7 +165,7 @@
           <a:bodyPr/>
           <a:p>
             <a:pPr>
-              <a:defRPr/>
+              <a:defRPr sz="1800"/>
             </a:pPr>
             <a:r>
               <a:t>DAU</a:t>
@@ -258,7 +258,7 @@
           <a:bodyPr/>
           <a:p>
             <a:pPr>
-              <a:defRPr/>
+              <a:defRPr sz="1800"/>
             </a:pPr>
             <a:r>
               <a:t>Revenue per day by variant (EUR)</a:t>
@@ -418,7 +418,7 @@
           <a:bodyPr/>
           <a:p>
             <a:pPr>
-              <a:defRPr/>
+              <a:defRPr sz="1800"/>
             </a:pPr>
             <a:r>
               <a:t>WAU</a:t>
@@ -509,7 +509,7 @@
           <a:bodyPr/>
           <a:p>
             <a:pPr>
-              <a:defRPr/>
+              <a:defRPr sz="1800"/>
             </a:pPr>
             <a:r>
               <a:t>MAU</a:t>
@@ -600,7 +600,7 @@
           <a:bodyPr/>
           <a:p>
             <a:pPr>
-              <a:defRPr/>
+              <a:defRPr sz="1800"/>
             </a:pPr>
             <a:r>
               <a:t>Revenue per day (EUR)</a:t>
@@ -693,10 +693,10 @@
           <a:bodyPr/>
           <a:p>
             <a:pPr>
-              <a:defRPr/>
+              <a:defRPr sz="1800"/>
             </a:pPr>
             <a:r>
-              <a:t>D1 retention by variant</a:t>
+              <a:t>Day-1 retention (%)</a:t>
             </a:r>
           </a:p>
         </rich>
@@ -28975,10 +28975,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
+  <dimension ref="A1:M32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1"/>
+    <row r="2"/>
+    <row r="17"/>
+    <row r="32"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>

</xml_diff>